<commit_message>
docs: deepen final report and rubric audit
</commit_message>
<xml_diff>
--- a/outputs/tables/tabelas_volatilidade_realizada_b3.xlsx
+++ b/outputs/tables/tabelas_volatilidade_realizada_b3.xlsx
@@ -538,19 +538,19 @@
         <v>60</v>
       </c>
       <c r="G2" t="n">
-        <v>4953</v>
+        <v>4952</v>
       </c>
       <c r="H2" t="n">
-        <v>82.55</v>
+        <v>82.53333333333333</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8598958333333333</v>
+        <v>0.9943775100401608</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2066960352422907</v>
+        <v>0.08028600612870269</v>
       </c>
       <c r="K2" t="n">
-        <v>0.990939125258292</v>
+        <v>0.9909367347438536</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -590,19 +590,19 @@
         <v>60</v>
       </c>
       <c r="G3" t="n">
-        <v>4955</v>
+        <v>4953</v>
       </c>
       <c r="H3" t="n">
-        <v>82.58333333333333</v>
+        <v>82.55</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8602430555555555</v>
+        <v>0.994578313253012</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1731853417899929</v>
+        <v>0.0418709150326797</v>
       </c>
       <c r="K3" t="n">
-        <v>0.990537523259468</v>
+        <v>0.9907335454434421</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -642,19 +642,19 @@
         <v>60</v>
       </c>
       <c r="G4" t="n">
-        <v>4960</v>
+        <v>4958</v>
       </c>
       <c r="H4" t="n">
-        <v>82.66666666666667</v>
+        <v>82.63333333333334</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8611111111111113</v>
+        <v>0.995582329317269</v>
       </c>
       <c r="J4" t="n">
-        <v>0.217215279000176</v>
+        <v>0.09283819628647209</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9901506140706846</v>
+        <v>0.9905426584386328</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -694,19 +694,19 @@
         <v>60</v>
       </c>
       <c r="G5" t="n">
-        <v>4949</v>
+        <v>4946</v>
       </c>
       <c r="H5" t="n">
-        <v>82.48333333333333</v>
+        <v>82.43333333333334</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8592013888888891</v>
+        <v>0.993172690763052</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3019932968777562</v>
+        <v>0.191041112701984</v>
       </c>
       <c r="K5" t="n">
-        <v>0.991950608818895</v>
+        <v>0.9919457111795572</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -752,10 +752,10 @@
         <v>82.18333333333334</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8560763888888888</v>
+        <v>0.9901606425702812</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2520339582596392</v>
+        <v>0.1323348379154698</v>
       </c>
       <c r="K6" t="n">
         <v>0.994551376236654</v>
@@ -798,19 +798,19 @@
         <v>60</v>
       </c>
       <c r="G7" t="n">
-        <v>4950</v>
+        <v>4949</v>
       </c>
       <c r="H7" t="n">
-        <v>82.5</v>
+        <v>82.48333333333333</v>
       </c>
       <c r="I7" t="n">
-        <v>0.8593750000000002</v>
+        <v>0.9937751004016064</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1891748942172073</v>
+        <v>0.0598937040065412</v>
       </c>
       <c r="K7" t="n">
-        <v>0.991551453372314</v>
+        <v>0.9915490628578756</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -856,10 +856,10 @@
         <v>82.59999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>0.8604166666666668</v>
+        <v>0.9951807228915662</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3381446928357683</v>
+        <v>0.2328096306876147</v>
       </c>
       <c r="K8" t="n">
         <v>0.991355666568714</v>
@@ -902,19 +902,19 @@
         <v>60</v>
       </c>
       <c r="G9" t="n">
-        <v>4941</v>
+        <v>4940</v>
       </c>
       <c r="H9" t="n">
-        <v>82.34999999999999</v>
+        <v>82.33333333333333</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8578125</v>
+        <v>0.9919678714859436</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2047299682315566</v>
+        <v>0.0777732296356938</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9911202775570817</v>
+        <v>0.9911178287374128</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -960,10 +960,10 @@
         <v>82.71666666666667</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8616319444444446</v>
+        <v>0.996586345381526</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4621198804710845</v>
+        <v>0.376655123243023</v>
       </c>
       <c r="K10" t="n">
         <v>0.988336271916936</v>
@@ -1006,19 +1006,19 @@
         <v>60</v>
       </c>
       <c r="G11" t="n">
-        <v>4944</v>
+        <v>4942</v>
       </c>
       <c r="H11" t="n">
-        <v>82.40000000000001</v>
+        <v>82.36666666666666</v>
       </c>
       <c r="I11" t="n">
-        <v>0.8583333333333333</v>
+        <v>0.9923694779116466</v>
       </c>
       <c r="J11" t="n">
-        <v>0.3466831333803811</v>
+        <v>0.242430441898527</v>
       </c>
       <c r="K11" t="n">
-        <v>0.9919357927040894</v>
+        <v>0.992337399129792</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1064,10 +1064,10 @@
         <v>82.58333333333333</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8602430555555557</v>
+        <v>0.9949799196787148</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5850615114235501</v>
+        <v>0.5191446028513238</v>
       </c>
       <c r="K12" t="n">
         <v>0.9805932815092064</v>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>precos parados 58.5% acima do maximo</t>
+          <t>precos parados 51.9% acima do maximo</t>
         </is>
       </c>
     </row>
@@ -1120,10 +1120,10 @@
         <v>82.53333333333333</v>
       </c>
       <c r="I13" t="n">
-        <v>0.8597222222222223</v>
+        <v>0.9943775100401606</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4517489892775532</v>
+        <v>0.3646363821552251</v>
       </c>
       <c r="K13" t="n">
         <v>0.9820343637422316</v>
@@ -1172,10 +1172,10 @@
         <v>82.61666666666666</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8605902777777779</v>
+        <v>0.9953815261044175</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5784934882083773</v>
+        <v>0.5114239086087311</v>
       </c>
       <c r="K14" t="n">
         <v>0.985498029455975</v>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>precos parados 57.8% acima do maximo</t>
+          <t>precos parados 51.1% acima do maximo</t>
         </is>
       </c>
     </row>
@@ -1442,28 +1442,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.448201818948554e-08</v>
+        <v>3.475337555231363e-08</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9906979709741012</v>
+        <v>0.990640680536115</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9906979709741012</v>
+        <v>0.990640680536115</v>
       </c>
       <c r="F4" t="n">
-        <v>-119.4183431355872</v>
+        <v>-119.6375983982553</v>
       </c>
       <c r="G4" t="n">
-        <v>246.8366862711744</v>
+        <v>247.2751967965107</v>
       </c>
       <c r="H4" t="n">
-        <v>255.1468360467973</v>
+        <v>255.5853465721336</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1632439953704395</v>
+        <v>0.1607494220984812</v>
       </c>
       <c r="J4" t="n">
         <v>59</v>
@@ -1502,7 +1502,7 @@
         <v>324.9245171046393</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3549874049094822</v>
+        <v>0.3549874049094821</v>
       </c>
       <c r="J5" t="n">
         <v>59</v>
@@ -1520,28 +1520,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.258114153094844e-08</v>
+        <v>3.358038936121591e-08</v>
       </c>
       <c r="C6" t="n">
-        <v>3.697693318668725e-11</v>
+        <v>9.625560666190219e-11</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9925637906288792</v>
+        <v>0.9925822893807322</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9925637906658562</v>
+        <v>0.9925822894769878</v>
       </c>
       <c r="F6" t="n">
-        <v>-117.4919310442452</v>
+        <v>-117.5169736115527</v>
       </c>
       <c r="G6" t="n">
-        <v>242.9838620884903</v>
+        <v>243.0339472231053</v>
       </c>
       <c r="H6" t="n">
-        <v>251.2940118641132</v>
+        <v>251.3440969987282</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1310067896993241</v>
+        <v>0.1310119040284162</v>
       </c>
       <c r="J6" t="n">
         <v>59</v>
@@ -1619,7 +1619,7 @@
         <v>322.6179587667132</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2342743840450768</v>
+        <v>0.2342743840450771</v>
       </c>
       <c r="J8" t="n">
         <v>59</v>
@@ -1715,28 +1715,28 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.226552007898682</v>
+        <v>2.226125547054353</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1746308859512775</v>
+        <v>0.1750972722234884</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1805739222307647</v>
+        <v>0.1802575428007602</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3552048081820422</v>
+        <v>0.3553548150242487</v>
       </c>
       <c r="F11" t="n">
-        <v>-119.3835928412744</v>
+        <v>-119.3797161231153</v>
       </c>
       <c r="G11" t="n">
-        <v>246.7671856825488</v>
+        <v>246.7594322462306</v>
       </c>
       <c r="H11" t="n">
-        <v>255.0773354581717</v>
+        <v>255.0695820218536</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.0411158269566819</v>
+        <v>-0.041094483635885</v>
       </c>
       <c r="J11" t="n">
         <v>59</v>
@@ -1874,40 +1874,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.764057301896003e-06</v>
+        <v>3.203960320765394e-06</v>
       </c>
       <c r="C2" t="n">
-        <v>0.001437642702498933</v>
+        <v>0.00154784320251154</v>
       </c>
       <c r="D2" t="n">
-        <v>1.221235463742723</v>
+        <v>1.133499470167432</v>
       </c>
       <c r="E2" t="n">
-        <v>18.62293307010334</v>
+        <v>15.65498546317322</v>
       </c>
       <c r="F2" t="n">
         <v>-0.008012435165124201</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.00395786471439736</v>
+        <v>-0.0041351141377288</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.0020484631956758</v>
+        <v>-0.0024126016353442</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0020554809157147</v>
+        <v>0.0024213640413273</v>
       </c>
       <c r="K2" t="n">
-        <v>0.004190129595182044</v>
+        <v>0.0043223096710844</v>
       </c>
       <c r="L2" t="n">
         <v>0.0227139482197693</v>
       </c>
       <c r="M2" t="n">
-        <v>5681</v>
+        <v>4901</v>
       </c>
     </row>
     <row r="3">
@@ -1917,40 +1917,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-2.964468740755564e-05</v>
+        <v>-3.438881054622889e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.002136177789995985</v>
+        <v>0.002300763551525544</v>
       </c>
       <c r="D3" t="n">
-        <v>0.124734159384027</v>
+        <v>0.122009534100117</v>
       </c>
       <c r="E3" t="n">
-        <v>4.683140709184015</v>
+        <v>3.625063011591902</v>
       </c>
       <c r="F3" t="n">
         <v>-0.0130806811758135</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.005955503905718721</v>
+        <v>-0.006037013315480159</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.0033465154203376</v>
+        <v>-0.003634688655054775</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.003313252783034413</v>
+        <v>0.003599362653126742</v>
       </c>
       <c r="K3" t="n">
-        <v>0.006327519250628281</v>
+        <v>0.006588395369528986</v>
       </c>
       <c r="L3" t="n">
         <v>0.0145497939167511</v>
       </c>
       <c r="M3" t="n">
-        <v>5654</v>
+        <v>4874</v>
       </c>
     </row>
     <row r="4">
@@ -1960,40 +1960,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-1.366005202477346e-05</v>
+        <v>-1.718934324917221e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.001449007225189259</v>
+        <v>0.001558512436837039</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0950416487760239</v>
+        <v>0.08835906611292567</v>
       </c>
       <c r="E4" t="n">
-        <v>5.535207324903045</v>
+        <v>4.374773989903566</v>
       </c>
       <c r="F4" t="n">
         <v>-0.0128239761662425</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.003936170280239652</v>
+        <v>-0.004051171729942268</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.00224541318067534</v>
+        <v>-0.00239452457338672</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.00226326441640516</v>
+        <v>0.002459991874876317</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0041400440991123</v>
+        <v>0.004500727602262847</v>
       </c>
       <c r="L4" t="n">
         <v>0.009254071542077</v>
       </c>
       <c r="M4" t="n">
-        <v>5669</v>
+        <v>4889</v>
       </c>
     </row>
     <row r="5">
@@ -2003,40 +2003,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.349962682374847e-05</v>
+        <v>2.723352556535038e-05</v>
       </c>
       <c r="C5" t="n">
-        <v>0.003595026369660208</v>
+        <v>0.003870152894373681</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7600136277448821</v>
+        <v>0.7031334986062513</v>
       </c>
       <c r="E5" t="n">
-        <v>6.845975040661276</v>
+        <v>5.494138531990591</v>
       </c>
       <c r="F5" t="n">
         <v>-0.0261608567866973</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.009359109823125716</v>
+        <v>-0.009776211998349292</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.005162698949509119</v>
+        <v>-0.0053619380003946</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0053908434383076</v>
+        <v>0.0056818280795707</v>
       </c>
       <c r="K5" t="n">
-        <v>0.01198653815777518</v>
+        <v>0.01253237391667242</v>
       </c>
       <c r="L5" t="n">
         <v>0.028104867639221</v>
       </c>
       <c r="M5" t="n">
-        <v>5689</v>
+        <v>4909</v>
       </c>
     </row>
     <row r="6">
@@ -2046,40 +2046,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-2.222107462631973e-05</v>
+        <v>-2.585895449300187e-05</v>
       </c>
       <c r="C6" t="n">
-        <v>0.001352339547635942</v>
+        <v>0.001455951297495219</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.5707608088197412</v>
+        <v>-0.5227202843894396</v>
       </c>
       <c r="E6" t="n">
-        <v>15.74441066656553</v>
+        <v>13.1695732751217</v>
       </c>
       <c r="F6" t="n">
         <v>-0.0215565554797656</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.00376016321246008</v>
+        <v>-0.003831898851291</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0021010898474003</v>
+        <v>-0.0022396464204099</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0020986402037959</v>
+        <v>0.0022722638338059</v>
       </c>
       <c r="K6" t="n">
-        <v>0.003775904707334157</v>
+        <v>0.0038635340507227</v>
       </c>
       <c r="L6" t="n">
         <v>0.0107688339522997</v>
       </c>
       <c r="M6" t="n">
-        <v>5681</v>
+        <v>4901</v>
       </c>
     </row>
     <row r="7">
@@ -2089,40 +2089,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.423481106123193e-05</v>
+        <v>1.649660625939059e-05</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003369325418401976</v>
+        <v>0.003627186272915917</v>
       </c>
       <c r="D7" t="n">
-        <v>0.001853211810024033</v>
+        <v>-0.0001498894375831869</v>
       </c>
       <c r="E7" t="n">
-        <v>7.746085898850071</v>
+        <v>6.273603240752352</v>
       </c>
       <c r="F7" t="n">
         <v>-0.0367237391971491</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.008165975563516776</v>
+        <v>-0.008230491061099901</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.0053050471972173</v>
+        <v>-0.0053619380003946</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0053476012130602</v>
+        <v>0.005399585380649751</v>
       </c>
       <c r="K7" t="n">
-        <v>0.01004045630779255</v>
+        <v>0.0105264030801237</v>
       </c>
       <c r="L7" t="n">
         <v>0.0262232273489588</v>
       </c>
       <c r="M7" t="n">
-        <v>5689</v>
+        <v>4909</v>
       </c>
     </row>
     <row r="8">
@@ -2132,40 +2132,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.0001274299104174022</v>
+        <v>-0.000147764470590392</v>
       </c>
       <c r="C8" t="n">
-        <v>0.002850152892704714</v>
+        <v>0.003068699090934309</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2567072994954627</v>
+        <v>0.2583910045384725</v>
       </c>
       <c r="E8" t="n">
-        <v>5.725598337044505</v>
+        <v>4.536811052797377</v>
       </c>
       <c r="F8" t="n">
         <v>-0.0191262480266249</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.008056189470309809</v>
+        <v>-0.008374379678313825</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.004545915724429144</v>
+        <v>-0.00475533471825383</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.004413310283101993</v>
+        <v>0.0045924264258156</v>
       </c>
       <c r="K8" t="n">
-        <v>0.008520743350609037</v>
+        <v>0.008826993219601162</v>
       </c>
       <c r="L8" t="n">
         <v>0.0216225295032057</v>
       </c>
       <c r="M8" t="n">
-        <v>5668</v>
+        <v>4888</v>
       </c>
     </row>
     <row r="9">
@@ -2175,40 +2175,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.427009441458573e-06</v>
+        <v>1.654398075644001e-06</v>
       </c>
       <c r="C9" t="n">
-        <v>0.001668232486133832</v>
+        <v>0.001796260136921322</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.03138657160118161</v>
+        <v>-0.02953107380601867</v>
       </c>
       <c r="E9" t="n">
-        <v>10.29129314544188</v>
+        <v>8.465629163500767</v>
       </c>
       <c r="F9" t="n">
         <v>-0.0150771780808423</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.00481671796723906</v>
+        <v>-0.005013332628638156</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0023374561029395</v>
+        <v>-0.00258342355535103</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.002313109114732832</v>
+        <v>0.002503970814388131</v>
       </c>
       <c r="K9" t="n">
-        <v>0.004959289626559312</v>
+        <v>0.005309894306669218</v>
       </c>
       <c r="L9" t="n">
         <v>0.0132862555874528</v>
       </c>
       <c r="M9" t="n">
-        <v>5675</v>
+        <v>4895</v>
       </c>
     </row>
     <row r="10">
@@ -2218,40 +2218,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-3.884201381989704e-05</v>
+        <v>-4.504274463846433e-05</v>
       </c>
       <c r="C10" t="n">
-        <v>0.002412639841906975</v>
+        <v>0.002598071996104682</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2443609727634594</v>
+        <v>0.2341047954194035</v>
       </c>
       <c r="E10" t="n">
-        <v>6.850498532523488</v>
+        <v>5.498077443247507</v>
       </c>
       <c r="F10" t="n">
         <v>-0.0209566883362004</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.00699339210479524</v>
+        <v>-0.00743267358955911</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.0037059930247571</v>
+        <v>-0.0039183553257357</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0.00382215977606265</v>
+        <v>0.004097093664678825</v>
       </c>
       <c r="K10" t="n">
-        <v>0.007225478942625283</v>
+        <v>0.007500665276839171</v>
       </c>
       <c r="L10" t="n">
         <v>0.0187840094357194</v>
       </c>
       <c r="M10" t="n">
-        <v>5666</v>
+        <v>4886</v>
       </c>
     </row>
     <row r="11">
@@ -2261,40 +2261,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.497708170867394e-07</v>
+        <v>6.388001358865029e-07</v>
       </c>
       <c r="C11" t="n">
-        <v>0.001404699780539869</v>
+        <v>0.001512479518248377</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.01130685344650456</v>
+        <v>-0.01067838190053868</v>
       </c>
       <c r="E11" t="n">
-        <v>6.206486966491825</v>
+        <v>4.942015345525149</v>
       </c>
       <c r="F11" t="n">
         <v>-0.0127044424515494</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.004019641708687875</v>
+        <v>-0.004103698373850125</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.00213844805212885</v>
+        <v>-0.00230159627305985</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.00217633014908085</v>
+        <v>0.00233160668559775</v>
       </c>
       <c r="K11" t="n">
-        <v>0.004461640452096</v>
+        <v>0.004727973138573704</v>
       </c>
       <c r="L11" t="n">
         <v>0.008150300833928901</v>
       </c>
       <c r="M11" t="n">
-        <v>5676</v>
+        <v>4896</v>
       </c>
     </row>
     <row r="12">
@@ -2304,40 +2304,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-9.805533764955129e-06</v>
+        <v>-1.136896719436335e-05</v>
       </c>
       <c r="C12" t="n">
-        <v>0.001810471995934218</v>
+        <v>0.001949493484583287</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1152906508853336</v>
+        <v>0.1094824850353144</v>
       </c>
       <c r="E12" t="n">
-        <v>5.156212607707271</v>
+        <v>4.035520803910646</v>
       </c>
       <c r="F12" t="n">
         <v>-0.0132529768069233</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.005167110953304396</v>
+        <v>-0.005315445670894973</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.002854993886589945</v>
+        <v>-0.003083268403755065</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.00290492156971498</v>
+        <v>0.003102626699221409</v>
       </c>
       <c r="K12" t="n">
-        <v>0.005263827427199961</v>
+        <v>0.005499754786448533</v>
       </c>
       <c r="L12" t="n">
         <v>0.0147970578116813</v>
       </c>
       <c r="M12" t="n">
-        <v>5672</v>
+        <v>4892</v>
       </c>
     </row>
   </sheetData>
@@ -2424,7 +2424,7 @@
         <v>0.01346113698242534</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2136889249180321</v>
+        <v>0.2136889249180322</v>
       </c>
       <c r="E2" t="n">
         <v>0.2094813730652876</v>
@@ -2439,10 +2439,10 @@
         <v>0.568335156447306</v>
       </c>
       <c r="I2" t="n">
-        <v>0.00017059413637498</v>
+        <v>0.0001708846895777735</v>
       </c>
       <c r="J2" t="n">
-        <v>2.907099587534861e-05</v>
+        <v>2.887801066723494e-05</v>
       </c>
       <c r="K2" t="n">
         <v>60</v>
@@ -2464,7 +2464,7 @@
         <v>0.3232331771254721</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3142676068187206</v>
+        <v>0.3142676068187207</v>
       </c>
       <c r="F3" t="n">
         <v>0.4130483756566108</v>
@@ -2476,10 +2476,10 @@
         <v>0.4663104139480986</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0004056452037798116</v>
+        <v>0.0004063431371817067</v>
       </c>
       <c r="J3" t="n">
-        <v>3.625093510059368e-05</v>
+        <v>3.580702132318902e-05</v>
       </c>
       <c r="K3" t="n">
         <v>60</v>
@@ -2492,16 +2492,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0001983619161130539</v>
+        <v>0.0001979034335859156</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01381951314567962</v>
+        <v>0.01380259656780732</v>
       </c>
       <c r="D4" t="n">
-        <v>0.219377970140738</v>
+        <v>0.2191094277922318</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2137360219540669</v>
+        <v>0.2108579694024383</v>
       </c>
       <c r="F4" t="n">
         <v>0.2782556742784386</v>
@@ -2510,13 +2510,13 @@
         <v>0.2948795544932061</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3392054485418272</v>
+        <v>0.3392054485418271</v>
       </c>
       <c r="I4" t="n">
-        <v>0.000182136049228933</v>
+        <v>0.0001821810060455399</v>
       </c>
       <c r="J4" t="n">
-        <v>1.787704694287435e-05</v>
+        <v>1.743345658426845e-05</v>
       </c>
       <c r="K4" t="n">
         <v>60</v>
@@ -2535,7 +2535,7 @@
         <v>0.03427357497800744</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5440761355976031</v>
+        <v>0.544076135597603</v>
       </c>
       <c r="E5" t="n">
         <v>0.5316491916625063</v>
@@ -2550,10 +2550,10 @@
         <v>0.986500274219542</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0009589509926479084</v>
+        <v>0.0009605791573304181</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0002698169029125235</v>
+        <v>0.0002682226765137994</v>
       </c>
       <c r="K5" t="n">
         <v>60</v>
@@ -2566,13 +2566,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0001731752589046208</v>
+        <v>0.0001731711452181592</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01279543964926507</v>
+        <v>0.01279526419032643</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2031213073661462</v>
+        <v>0.2031185220418443</v>
       </c>
       <c r="E6" t="n">
         <v>0.1872670179976995</v>
@@ -2587,10 +2587,10 @@
         <v>0.442378595010617</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0001642118013703933</v>
+        <v>0.0001644915299737587</v>
       </c>
       <c r="J6" t="n">
-        <v>1.433316652392411e-05</v>
+        <v>1.417082905505455e-05</v>
       </c>
       <c r="K6" t="n">
         <v>60</v>
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00107622235056501</v>
+        <v>0.001076222350565011</v>
       </c>
       <c r="C7" t="n">
         <v>0.03207838395824941</v>
@@ -2624,10 +2624,10 @@
         <v>0.9109821496128452</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00086384238878419</v>
+        <v>0.0008653077054074101</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0002140607621812309</v>
+        <v>0.0002127801818699186</v>
       </c>
       <c r="K7" t="n">
         <v>60</v>
@@ -2658,13 +2658,13 @@
         <v>0.6030916761176272</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8142270724495367</v>
+        <v>0.8142270724495366</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0006816786955852466</v>
+        <v>0.0006828460745085217</v>
       </c>
       <c r="J8" t="n">
-        <v>9.026290649632861e-05</v>
+        <v>8.924270841767506e-05</v>
       </c>
       <c r="K8" t="n">
         <v>60</v>
@@ -2686,7 +2686,7 @@
         <v>0.2486917177041878</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2321490300740516</v>
+        <v>0.2321490300740517</v>
       </c>
       <c r="F9" t="n">
         <v>0.3305899767876974</v>
@@ -2698,10 +2698,10 @@
         <v>0.4566446077757097</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0002352981127023958</v>
+        <v>0.0002357007478897834</v>
       </c>
       <c r="J9" t="n">
-        <v>3.073743438055852e-05</v>
+        <v>3.045372115719123e-05</v>
       </c>
       <c r="K9" t="n">
         <v>60</v>
@@ -2735,10 +2735,10 @@
         <v>0.6746095503147842</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0004832260436550517</v>
+        <v>0.0004840544047129767</v>
       </c>
       <c r="J10" t="n">
-        <v>7.081901298241362e-05</v>
+        <v>7.017671345502778e-05</v>
       </c>
       <c r="K10" t="n">
         <v>60</v>
@@ -2751,19 +2751,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0001866301096229735</v>
+        <v>0.0001866296010452185</v>
       </c>
       <c r="C11" t="n">
-        <v>0.01344476962889574</v>
+        <v>0.01344475012427417</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2134291012356745</v>
+        <v>0.213428791609406</v>
       </c>
       <c r="E11" t="n">
         <v>0.2079028832598891</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2665587521060798</v>
+        <v>0.2665587521060797</v>
       </c>
       <c r="G11" t="n">
         <v>0.2773442794584063</v>
@@ -2772,10 +2772,10 @@
         <v>0.3358024539460292</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0001739360410640366</v>
+        <v>0.0001742290721413719</v>
       </c>
       <c r="J11" t="n">
-        <v>1.582445247942295e-05</v>
+        <v>1.561875744291574e-05</v>
       </c>
       <c r="K11" t="n">
         <v>60</v>
@@ -2803,16 +2803,16 @@
         <v>0.330466675557028</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3749122145089814</v>
+        <v>0.3749122145089815</v>
       </c>
       <c r="H12" t="n">
         <v>0.4990499834037444</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0002899332437701427</v>
+        <v>0.0002904291099983995</v>
       </c>
       <c r="J12" t="n">
-        <v>2.521187317415431e-05</v>
+        <v>2.492466545752003e-05</v>
       </c>
       <c r="K12" t="n">
         <v>60</v>
@@ -2890,16 +2890,16 @@
         <v>0.1666666666666667</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1156776355389515</v>
+        <v>0.1146548736162371</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4775645446393343</v>
+        <v>0.4766613982404395</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="H2" t="n">
-        <v>5.384753441595894</v>
+        <v>4.987258230282089</v>
       </c>
     </row>
     <row r="3">
@@ -2918,16 +2918,16 @@
         <v>0.08333333333333333</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08042574779886276</v>
+        <v>0.07938851548807462</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3778907269318962</v>
+        <v>0.3768152720715392</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46140</v>
       </c>
       <c r="H3" t="n">
-        <v>3.996129442744163</v>
+        <v>3.983739523761189</v>
       </c>
     </row>
     <row r="4">
@@ -2940,22 +2940,22 @@
         <v>60</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1166666666666667</v>
       </c>
       <c r="E4" t="n">
-        <v>0.09805943816618873</v>
+        <v>0.09589164513886532</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3491843490077225</v>
+        <v>0.3480327764661545</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="H4" t="n">
-        <v>3.768387892335181</v>
+        <v>3.755881111393931</v>
       </c>
     </row>
     <row r="5">
@@ -2968,22 +2968,22 @@
         <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3833333333333334</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2164084973902562</v>
+        <v>0.2151071368619721</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4758797593941737</v>
+        <v>0.4749943060962041</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46169</v>
       </c>
       <c r="H5" t="n">
-        <v>5.364765851062979</v>
+        <v>5.340835103423853</v>
       </c>
     </row>
     <row r="6">
@@ -3002,16 +3002,16 @@
         <v>0.05</v>
       </c>
       <c r="E6" t="n">
-        <v>0.06826701015488883</v>
+        <v>0.06730781711501523</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2961000082258066</v>
+        <v>0.2948831598357714</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="H6" t="n">
-        <v>2.734741360543586</v>
+        <v>2.722696140073457</v>
       </c>
     </row>
     <row r="7">
@@ -3024,22 +3024,22 @@
         <v>60</v>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.35</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1906484510452018</v>
+        <v>0.1894728931692779</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5498922298445653</v>
+        <v>0.5491318138585979</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46147</v>
       </c>
       <c r="H7" t="n">
-        <v>5.145197454129557</v>
+        <v>4.768684289284589</v>
       </c>
     </row>
     <row r="8">
@@ -3052,22 +3052,22 @@
         <v>60</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1166666666666667</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1193025554641736</v>
+        <v>0.1180236511582866</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4342680702833554</v>
+        <v>0.433312317835491</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46129</v>
       </c>
       <c r="H8" t="n">
-        <v>4.245214522801748</v>
+        <v>4.235788382198122</v>
       </c>
     </row>
     <row r="9">
@@ -3080,22 +3080,22 @@
         <v>60</v>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1245211845587535</v>
+        <v>0.1234136589578279</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4204948110066509</v>
+        <v>0.4195157898946414</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="H9" t="n">
-        <v>4.789442792451213</v>
+        <v>4.778197958561689</v>
       </c>
     </row>
     <row r="10">
@@ -3114,16 +3114,16 @@
         <v>0.1666666666666667</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1300314200090638</v>
+        <v>0.1288290679790122</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6078365774731502</v>
+        <v>0.6071740531725851</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>46108</v>
       </c>
       <c r="H10" t="n">
-        <v>5.851878616825123</v>
+        <v>5.845385528413154</v>
       </c>
     </row>
     <row r="11">
@@ -3142,16 +3142,16 @@
         <v>0.03333333333333333</v>
       </c>
       <c r="E11" t="n">
-        <v>0.07950648352357774</v>
+        <v>0.07840907976026282</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3221159799353333</v>
+        <v>0.3209707567695323</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="H11" t="n">
-        <v>3.870020778118747</v>
+        <v>3.724482801952026</v>
       </c>
     </row>
     <row r="12">
@@ -3170,16 +3170,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0748758689829807</v>
+        <v>0.07395143985769394</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3382637311669217</v>
+        <v>0.3371197721915456</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="H12" t="n">
-        <v>4.202550517136237</v>
+        <v>3.887946812201539</v>
       </c>
     </row>
   </sheetData>
@@ -3246,16 +3246,16 @@
         <v>480</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01620323725970493</v>
+        <v>0.01620109831702586</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2572184173401304</v>
+        <v>0.2571844626777458</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1166666666666667</v>
+        <v>0.1104166666666667</v>
       </c>
       <c r="G2" t="n">
-        <v>0.09642059859165844</v>
+        <v>0.09523076223912362</v>
       </c>
     </row>
     <row r="3">
@@ -3277,10 +3277,10 @@
         <v>0.4938749805531023</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2888888888888889</v>
+        <v>0.2722222222222222</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1754531679665439</v>
+        <v>0.1742012270631788</v>
       </c>
     </row>
   </sheetData>
@@ -3361,13 +3361,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5440761355976031</v>
+        <v>0.544076135597603</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3833333333333334</v>
+        <v>0.3666666666666666</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2164084973902562</v>
+        <v>0.2151071368619721</v>
       </c>
       <c r="E2" t="n">
         <v>0.868914012766817</v>
@@ -3405,10 +3405,10 @@
         <v>0.5092285584862309</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3666666666666666</v>
+        <v>0.35</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1906484510452018</v>
+        <v>0.1894728931692779</v>
       </c>
       <c r="E3" t="n">
         <v>0.9931310652892432</v>
@@ -3446,10 +3446,10 @@
         <v>0.4283202475754732</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1166666666666667</v>
+        <v>0.1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1193025554641736</v>
+        <v>0.1180236511582866</v>
       </c>
       <c r="E4" t="n">
         <v>0.5019277823564871</v>
@@ -3490,7 +3490,7 @@
         <v>0.1666666666666667</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1300314200090638</v>
+        <v>0.1288290679790122</v>
       </c>
       <c r="E5" t="n">
         <v>0.999999995829248</v>
@@ -3531,7 +3531,7 @@
         <v>0.08333333333333333</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08042574779886276</v>
+        <v>0.07938851548807462</v>
       </c>
       <c r="E6" t="n">
         <v>0.919203512490246</v>
@@ -3572,7 +3572,7 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0748758689829807</v>
+        <v>0.07395143985769394</v>
       </c>
       <c r="E7" t="n">
         <v>0.0166284019084208</v>
@@ -3586,7 +3586,7 @@
         <v>6</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I7" t="n">
         <v>10</v>
@@ -3610,10 +3610,10 @@
         <v>0.2486917177041878</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1245211845587535</v>
+        <v>0.1234136589578279</v>
       </c>
       <c r="E8" t="n">
         <v>0.9795049375808044</v>
@@ -3627,7 +3627,7 @@
         <v>7</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I8" t="n">
         <v>4</v>
@@ -3648,16 +3648,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.219377970140738</v>
+        <v>0.2191094277922318</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1166666666666667</v>
       </c>
       <c r="D9" t="n">
-        <v>0.09805943816618873</v>
+        <v>0.09589164513886532</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9906979709741012</v>
+        <v>0.990640680536115</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -3668,7 +3668,7 @@
         <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I9" t="n">
         <v>7</v>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>volatilidade abaixo da mediana; maior incidencia relativa de jumps; grupo core_liquid</t>
+          <t>volatilidade abaixo da mediana; menor incidencia relativa de jumps; grupo core_liquid</t>
         </is>
       </c>
     </row>
@@ -3689,13 +3689,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2136889249180321</v>
+        <v>0.2136889249180322</v>
       </c>
       <c r="C10" t="n">
         <v>0.1666666666666667</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1156776355389515</v>
+        <v>0.1146548736162371</v>
       </c>
       <c r="E10" t="n">
         <v>0.9417503331908312</v>
@@ -3730,16 +3730,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2134291012356745</v>
+        <v>0.213428791609406</v>
       </c>
       <c r="C11" t="n">
         <v>0.03333333333333333</v>
       </c>
       <c r="D11" t="n">
-        <v>0.07950648352357774</v>
+        <v>0.07840907976026282</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3552048081820422</v>
+        <v>0.3553548150242487</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -3771,16 +3771,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2031213073661462</v>
+        <v>0.2031185220418443</v>
       </c>
       <c r="C12" t="n">
         <v>0.05</v>
       </c>
       <c r="D12" t="n">
-        <v>0.06826701015488883</v>
+        <v>0.06730781711501523</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9925637906658562</v>
+        <v>0.9925822894769878</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>

</xml_diff>